<commit_message>
Classify Smart Wash Laundry as Services
Recategorises the Dec 2020 SMART WASH LAUNDRY transaction from Other to a
new Services category in the master workbook (Notes sheet updated) and
regenerates data/spend-rates.json. The donut draws Services as hatched
green, placed between Pharmacy and Supermarket so neighbouring slices stay
distinguishable. Spend rates are unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NBtxQTve9NxEq7k6UrG86P
</commit_message>
<xml_diff>
--- a/data/Master_Data_V0.1.xlsx
+++ b/data/Master_Data_V0.1.xlsx
@@ -5861,7 +5861,7 @@
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Services</t>
         </is>
       </c>
       <c r="G183" s="4" t="str">
@@ -18592,7 +18592,7 @@
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Transactions that fit none of the 8 categories (car dealer/service, gym, tax prep, donation, zoo/Top Golf/tickets, medical, barber, laundry, government fees, Costco membership) are labelled "Other".</t>
+          <t>Transactions that fit none of the 8 categories (car dealer/service, gym, tax prep, donation, zoo/Top Golf/tickets, medical, barber, government fees, Costco membership) are labelled "Other". Laundry (Smart Wash Laundry) is labelled "Services".</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Categorise Target as Supermarket / Groceries
Moves all 28 Target transactions (six stores, including two refunds) from
Merchandise / Clothing to Supermarket / Groceries in the master workbook and
regenerates data/spend-rates.json. Spend rates are unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NBtxQTve9NxEq7k6UrG86P
</commit_message>
<xml_diff>
--- a/data/Master_Data_V0.1.xlsx
+++ b/data/Master_Data_V0.1.xlsx
@@ -3137,7 +3137,7 @@
         <v>8.98</v>
       </c>
       <c r="F88" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G88" s="4" t="str">
         <f>IF(F88="Payment / Credit","Payment",IF(E88&lt;0,"Income","Spend"))</f>
@@ -4505,7 +4505,7 @@
         <v>45.37</v>
       </c>
       <c r="F145" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G145" s="4" t="str">
         <f>IF(F145="Payment / Credit","Payment",IF(E145&lt;0,"Income","Spend"))</f>
@@ -4577,7 +4577,7 @@
         <v>17.64</v>
       </c>
       <c r="F148" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G148" s="4" t="str">
         <f>IF(F148="Payment / Credit","Payment",IF(E148&lt;0,"Income","Spend"))</f>
@@ -4625,7 +4625,7 @@
         <v>88.17</v>
       </c>
       <c r="F150" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G150" s="4" t="str">
         <f>IF(F150="Payment / Credit","Payment",IF(E150&lt;0,"Income","Spend"))</f>
@@ -4841,7 +4841,7 @@
         <v>85.65</v>
       </c>
       <c r="F159" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G159" s="4" t="str">
         <f>IF(F159="Payment / Credit","Payment",IF(E159&lt;0,"Income","Spend"))</f>
@@ -5153,7 +5153,7 @@
         <v>13.95</v>
       </c>
       <c r="F172" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G172" s="4" t="str">
         <f>IF(F172="Payment / Credit","Payment",IF(E172&lt;0,"Income","Spend"))</f>
@@ -5921,7 +5921,7 @@
         <v>3.3</v>
       </c>
       <c r="F204" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G204" s="4" t="str">
         <f>IF(F204="Payment / Credit","Payment",IF(E204&lt;0,"Income","Spend"))</f>
@@ -6569,7 +6569,7 @@
         <v>3.05</v>
       </c>
       <c r="F231" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G231" s="4" t="str">
         <f>IF(F231="Payment / Credit","Payment",IF(E231&lt;0,"Income","Spend"))</f>
@@ -8777,7 +8777,7 @@
         <v>20.85</v>
       </c>
       <c r="F323" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G323" s="4" t="str">
         <f>IF(F323="Payment / Credit","Payment",IF(E323&lt;0,"Income","Spend"))</f>
@@ -9137,7 +9137,7 @@
         <v>5.72</v>
       </c>
       <c r="F338" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G338" s="4" t="str">
         <f>IF(F338="Payment / Credit","Payment",IF(E338&lt;0,"Income","Spend"))</f>
@@ -9425,7 +9425,7 @@
         <v>20.350000000000001</v>
       </c>
       <c r="F350" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G350" s="4" t="str">
         <f>IF(F350="Payment / Credit","Payment",IF(E350&lt;0,"Income","Spend"))</f>
@@ -9761,7 +9761,7 @@
         <v>23.13</v>
       </c>
       <c r="F364" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G364" s="4" t="str">
         <f>IF(F364="Payment / Credit","Payment",IF(E364&lt;0,"Income","Spend"))</f>
@@ -9809,7 +9809,7 @@
         <v>36.71</v>
       </c>
       <c r="F366" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G366" s="4" t="str">
         <f>IF(F366="Payment / Credit","Payment",IF(E366&lt;0,"Income","Spend"))</f>
@@ -10361,7 +10361,7 @@
         <v>19.190000000000001</v>
       </c>
       <c r="F389" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G389" s="4" t="str">
         <f>IF(F389="Payment / Credit","Payment",IF(E389&lt;0,"Income","Spend"))</f>
@@ -11249,7 +11249,7 @@
         <v>9.7899999999999991</v>
       </c>
       <c r="F426" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G426" s="4" t="str">
         <f>IF(F426="Payment / Credit","Payment",IF(E426&lt;0,"Income","Spend"))</f>
@@ -11465,7 +11465,7 @@
         <v>41.63</v>
       </c>
       <c r="F435" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G435" s="4" t="str">
         <f>IF(F435="Payment / Credit","Payment",IF(E435&lt;0,"Income","Spend"))</f>
@@ -11489,7 +11489,7 @@
         <v>13.25</v>
       </c>
       <c r="F436" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G436" s="4" t="str">
         <f>IF(F436="Payment / Credit","Payment",IF(E436&lt;0,"Income","Spend"))</f>
@@ -11633,7 +11633,7 @@
         <v>30.24</v>
       </c>
       <c r="F442" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G442" s="4" t="str">
         <f>IF(F442="Payment / Credit","Payment",IF(E442&lt;0,"Income","Spend"))</f>
@@ -11777,7 +11777,7 @@
         <v>-2.86</v>
       </c>
       <c r="F448" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G448" s="4" t="str">
         <f>IF(F448="Payment / Credit","Payment",IF(E448&lt;0,"Income","Spend"))</f>
@@ -11801,7 +11801,7 @@
         <v>10.77</v>
       </c>
       <c r="F449" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G449" s="4" t="str">
         <f>IF(F449="Payment / Credit","Payment",IF(E449&lt;0,"Income","Spend"))</f>
@@ -11825,7 +11825,7 @@
         <v>23.78</v>
       </c>
       <c r="F450" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G450" s="4" t="str">
         <f>IF(F450="Payment / Credit","Payment",IF(E450&lt;0,"Income","Spend"))</f>
@@ -12113,7 +12113,7 @@
         <v>18.73</v>
       </c>
       <c r="F462" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G462" s="4" t="str">
         <f>IF(F462="Payment / Credit","Payment",IF(E462&lt;0,"Income","Spend"))</f>
@@ -12329,7 +12329,7 @@
         <v>3.66</v>
       </c>
       <c r="F471" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G471" s="4" t="str">
         <f>IF(F471="Payment / Credit","Payment",IF(E471&lt;0,"Income","Spend"))</f>
@@ -13265,7 +13265,7 @@
         <v>3.35</v>
       </c>
       <c r="F510" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G510" s="4" t="str">
         <f>IF(F510="Payment / Credit","Payment",IF(E510&lt;0,"Income","Spend"))</f>
@@ -13385,7 +13385,7 @@
         <v>4.79</v>
       </c>
       <c r="F515" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G515" s="4" t="str">
         <f>IF(F515="Payment / Credit","Payment",IF(E515&lt;0,"Income","Spend"))</f>
@@ -13697,7 +13697,7 @@
         <v>57.59</v>
       </c>
       <c r="F528" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G528" s="4" t="str">
         <f>IF(F528="Payment / Credit","Payment",IF(E528&lt;0,"Income","Spend"))</f>
@@ -13817,7 +13817,7 @@
         <v>68.53</v>
       </c>
       <c r="F533" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G533" s="4" t="str">
         <f>IF(F533="Payment / Credit","Payment",IF(E533&lt;0,"Income","Spend"))</f>
@@ -13937,7 +13937,7 @@
         <v>-38.58</v>
       </c>
       <c r="F538" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G538" s="4" t="str">
         <f>IF(F538="Payment / Credit","Payment",IF(E538&lt;0,"Income","Spend"))</f>

</xml_diff>